<commit_message>
fix: only take assignment once for every id value
</commit_message>
<xml_diff>
--- a/inst/extdata/Verbatims_fake_survey.xlsx
+++ b/inst/extdata/Verbatims_fake_survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Codestufen" sheetId="1" state="visible" r:id="rId2"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="114">
   <si>
     <t xml:space="preserve">love </t>
   </si>
@@ -425,6 +425,12 @@
     <t xml:space="preserve">Calc3 Zuord 10</t>
   </si>
   <si>
+    <t xml:space="preserve">q6_test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THIS id value is not in the data!!!</t>
+  </si>
+  <si>
     <t xml:space="preserve">q6mcg</t>
   </si>
 </sst>
@@ -667,7 +673,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -795,6 +801,10 @@
     <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -19009,7 +19019,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BD132"/>
+  <dimension ref="A1:BD134"/>
   <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="11.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="3" min="1" style="7" width="11.52"/>
@@ -28389,8 +28399,32 @@
       <c r="BC132" s="29"/>
       <c r="BD132" s="29"/>
     </row>
+    <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D133" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E133" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G133" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H133" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D134" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E134" s="7" t="n">
+        <v>9999999</v>
+      </c>
+      <c r="F134" s="32" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
-  <sheetProtection sheet="true" objects="true" scenarios="true" formatCells="false" formatColumns="false" formatRows="false" sort="false" autoFilter="false"/>
   <autoFilter ref="D32:BD132"/>
   <mergeCells count="2">
     <mergeCell ref="H11:J14"/>
@@ -28447,7 +28481,7 @@
         <v>31</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E1" s="9"/>
       <c r="F1" s="10"/>

</xml_diff>